<commit_message>
vault backup: 2026-10-10 11:31:03
</commit_message>
<xml_diff>
--- a/module_10/Module 10.xlsx
+++ b/module_10/Module 10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamheier/Documents/Auslandssemester/Kurse/ict-702-data-visualisation/module_10/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8EF08B7-1AF8-694E-B551-675663BB888E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9671D97B-8025-6F4A-B6CF-F729D878F3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="2" xr2:uid="{C543A414-E662-4178-8E39-C55C3D99B4E3}"/>
   </bookViews>
@@ -17,34 +17,6 @@
     <sheet name="PositiveOhioChart" sheetId="4" r:id="rId2"/>
     <sheet name="MaximusFashionChart" sheetId="5" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">MaximusFashionChart!$B$1</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">MaximusFashionChart!$B$2:$B$9</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">MaximusFashionChart!$B$1</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">MaximusFashionChart!$B$2:$B$9</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">MaximusFashionChart!$B$1</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">MaximusFashionChart!$B$2:$B$9</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">MaximusFashionChart!$B$1</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">MaximusFashionChart!$B$2:$B$9</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">MaximusFashionChart!$B$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">MaximusFashionChart!$B$2:$B$9</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">MaximusFashionChart!$C$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">MaximusFashionChart!$C$2:$C$9</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -7128,6 +7100,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="465554495"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -17532,28 +17505,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="53d19f74-6bc9-4aed-b277-f53d52e7cc56" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e88296c4-2d3a-4b5e-b7cc-73362ec365d5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000E01F302C440524FA31D7DCD25615BF1" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="541c2a5d964e9a5d7d5542e305e11e77">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="e88296c4-2d3a-4b5e-b7cc-73362ec365d5" xmlns:ns3="53d19f74-6bc9-4aed-b277-f53d52e7cc56" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="01a55807868fe61ce416780883e98636" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -17813,10 +17764,44 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="53d19f74-6bc9-4aed-b277-f53d52e7cc56" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e88296c4-2d3a-4b5e-b7cc-73362ec365d5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6191F80-060B-4806-85FA-2C5706CA4F8A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{899B41A2-6226-4E7E-B848-7ADAA4611474}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="e88296c4-2d3a-4b5e-b7cc-73362ec365d5"/>
+    <ds:schemaRef ds:uri="53d19f74-6bc9-4aed-b277-f53d52e7cc56"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17834,21 +17819,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{899B41A2-6226-4E7E-B848-7ADAA4611474}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6191F80-060B-4806-85FA-2C5706CA4F8A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="e88296c4-2d3a-4b5e-b7cc-73362ec365d5"/>
-    <ds:schemaRef ds:uri="53d19f74-6bc9-4aed-b277-f53d52e7cc56"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-15 12:02:35
</commit_message>
<xml_diff>
--- a/module_10/Module 10.xlsx
+++ b/module_10/Module 10.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamheier/Documents/Auslandssemester/Kurse/ict-702-data-visualisation/module_10/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9671D97B-8025-6F4A-B6CF-F729D878F3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74680239-B44A-AD49-BDB8-0283B08FF741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="2" xr2:uid="{C543A414-E662-4178-8E39-C55C3D99B4E3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="3" xr2:uid="{C543A414-E662-4178-8E39-C55C3D99B4E3}"/>
   </bookViews>
   <sheets>
-    <sheet name="GuaraldiConsultants" sheetId="2" r:id="rId1"/>
-    <sheet name="PositiveOhioChart" sheetId="4" r:id="rId2"/>
-    <sheet name="MaximusFashionChart" sheetId="5" r:id="rId3"/>
+    <sheet name="JavaCup" sheetId="6" r:id="rId1"/>
+    <sheet name="GuaraldiConsultants" sheetId="2" r:id="rId2"/>
+    <sheet name="PositiveOhioChart" sheetId="4" r:id="rId3"/>
+    <sheet name="MaximusFashionChart" sheetId="5" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">JavaCup!$A$1:$F$218</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="16">
   <si>
     <t>Years of Service</t>
   </si>
@@ -67,6 +71,24 @@
   <si>
     <t>Quarter</t>
   </si>
+  <si>
+    <t>Depth of the Chocolate Flavor of the Cup</t>
+  </si>
+  <si>
+    <t>Sweetness</t>
+  </si>
+  <si>
+    <t>Creaminess of Filling</t>
+  </si>
+  <si>
+    <t>Texture</t>
+  </si>
+  <si>
+    <t>Taste</t>
+  </si>
+  <si>
+    <t>Respondent</t>
+  </si>
 </sst>
 </file>
 
@@ -78,9 +100,16 @@
     <numFmt numFmtId="166" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +125,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,23 +158,44 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -288,7 +346,7 @@
             <c:numRef>
               <c:f>GuaraldiConsultants!$A$2:$A$112</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>#,#00</c:formatCode>
                 <c:ptCount val="111"/>
                 <c:pt idx="0">
                   <c:v>2.5</c:v>
@@ -630,7 +688,7 @@
             <c:numRef>
               <c:f>GuaraldiConsultants!$B$2:$B$112</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>#,#00</c:formatCode>
                 <c:ptCount val="111"/>
                 <c:pt idx="0">
                   <c:v>18</c:v>
@@ -1064,7 +1122,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="#,#00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1181,7 +1239,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="#,#00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1333,10 +1391,10 @@
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>7,5</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>76,0</c:v>
+                  <c:v>76.0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2017,7 +2075,7 @@
             <c:numRef>
               <c:f>GuaraldiConsultants!$A$2:$A$57</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>#,#00</c:formatCode>
                 <c:ptCount val="56"/>
                 <c:pt idx="0">
                   <c:v>2.5</c:v>
@@ -2194,7 +2252,7 @@
             <c:numRef>
               <c:f>GuaraldiConsultants!$B$2:$B$57</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>#,#00</c:formatCode>
                 <c:ptCount val="56"/>
                 <c:pt idx="0">
                   <c:v>18</c:v>
@@ -2406,7 +2464,7 @@
             <c:numRef>
               <c:f>GuaraldiConsultants!$A$58:$A$112</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>#,#00</c:formatCode>
                 <c:ptCount val="55"/>
                 <c:pt idx="0">
                   <c:v>3</c:v>
@@ -2580,7 +2638,7 @@
             <c:numRef>
               <c:f>GuaraldiConsultants!$B$58:$B$112</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>#,#00</c:formatCode>
                 <c:ptCount val="55"/>
                 <c:pt idx="0">
                   <c:v>65</c:v>
@@ -2844,7 +2902,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="#,#00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2964,7 +3022,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="#,#00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3851,7 +3909,7 @@
             <c:numRef>
               <c:f>PositiveOhioChart!$B$2:$B$205</c:f>
               <c:numCache>
-                <c:formatCode>0.0%</c:formatCode>
+                <c:formatCode>#,#00%</c:formatCode>
                 <c:ptCount val="204"/>
                 <c:pt idx="0">
                   <c:v>8.6224990690273881E-2</c:v>
@@ -4539,7 +4597,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="0.0%" sourceLinked="1"/>
+        <c:numFmt formatCode="#,#00%" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -5375,7 +5433,7 @@
             <c:numRef>
               <c:f>PositiveOhioChart!$B$2:$B$205</c:f>
               <c:numCache>
-                <c:formatCode>0.0%</c:formatCode>
+                <c:formatCode>#,#00%</c:formatCode>
                 <c:ptCount val="204"/>
                 <c:pt idx="0">
                   <c:v>8.6224990690273881E-2</c:v>
@@ -6078,7 +6136,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.0%" sourceLinked="1"/>
+        <c:numFmt formatCode="#,#00%" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -6429,7 +6487,7 @@
             <c:numRef>
               <c:f>MaximusFashionChart!$C$2:$C$9</c:f>
               <c:numCache>
-                <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_(* #.##0_);_(* \(#.##0\);_(* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>815000</c:v>
@@ -6908,7 +6966,7 @@
             <c:numRef>
               <c:f>MaximusFashionChart!$C$2:$C$9</c:f>
               <c:numCache>
-                <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_(* #.##0_);_(* \(#.##0\);_(* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>815000</c:v>
@@ -7053,7 +7111,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="r"/>
-        <c:numFmt formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:numFmt formatCode="_(* #.##0_);_(* \(#.##0\);_(* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -7717,6 +7775,7 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -7724,6 +7783,7 @@
                 </c:ext>
               </c:extLst>
             </c:dLbl>
+            <c:numFmt formatCode="#,##0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -7760,6 +7820,7 @@
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
+            <c:separator>, </c:separator>
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -7785,7 +7846,7 @@
             <c:numRef>
               <c:f>MaximusFashionChart!$C$2:$C$9</c:f>
               <c:numCache>
-                <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_(* #.##0_);_(* \(#.##0\);_(* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>815000</c:v>
@@ -7998,7 +8059,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:numFmt formatCode="_(* #.##0_);_(* \(#.##0\);_(* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -14402,6 +14463,4406 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7031D5CB-845F-C443-A959-7B57D41E4497}">
+  <dimension ref="A1:F220"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9.1640625" style="9"/>
+    <col min="4" max="4" width="12.6640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="11.5" style="9" customWidth="1"/>
+    <col min="6" max="6" width="22.1640625" style="9" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="12">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11">
+        <v>42</v>
+      </c>
+      <c r="C2" s="11">
+        <v>76</v>
+      </c>
+      <c r="D2" s="11">
+        <v>92</v>
+      </c>
+      <c r="E2" s="11">
+        <v>86</v>
+      </c>
+      <c r="F2" s="11">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="12">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11">
+        <v>32</v>
+      </c>
+      <c r="C3" s="11">
+        <v>94</v>
+      </c>
+      <c r="D3" s="11">
+        <v>98</v>
+      </c>
+      <c r="E3" s="11">
+        <v>72</v>
+      </c>
+      <c r="F3" s="11">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="12">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11">
+        <v>32</v>
+      </c>
+      <c r="C4" s="11">
+        <v>99</v>
+      </c>
+      <c r="D4" s="11">
+        <v>79</v>
+      </c>
+      <c r="E4" s="11">
+        <v>71</v>
+      </c>
+      <c r="F4" s="11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="12">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11">
+        <v>48</v>
+      </c>
+      <c r="C5" s="11">
+        <v>70</v>
+      </c>
+      <c r="D5" s="11">
+        <v>59</v>
+      </c>
+      <c r="E5" s="11">
+        <v>44</v>
+      </c>
+      <c r="F5" s="11">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="12">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11">
+        <v>64</v>
+      </c>
+      <c r="C6" s="11">
+        <v>97</v>
+      </c>
+      <c r="D6" s="11">
+        <v>75</v>
+      </c>
+      <c r="E6" s="11">
+        <v>59</v>
+      </c>
+      <c r="F6" s="11">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="12">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11">
+        <v>96</v>
+      </c>
+      <c r="C7" s="11">
+        <v>71</v>
+      </c>
+      <c r="D7" s="11">
+        <v>88</v>
+      </c>
+      <c r="E7" s="11">
+        <v>66</v>
+      </c>
+      <c r="F7" s="11">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="12">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11">
+        <v>56</v>
+      </c>
+      <c r="C8" s="11">
+        <v>75</v>
+      </c>
+      <c r="D8" s="11">
+        <v>99</v>
+      </c>
+      <c r="E8" s="11">
+        <v>93</v>
+      </c>
+      <c r="F8" s="11">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="12">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11">
+        <v>72</v>
+      </c>
+      <c r="C9" s="11">
+        <v>52</v>
+      </c>
+      <c r="D9" s="11">
+        <v>100</v>
+      </c>
+      <c r="E9" s="11">
+        <v>61</v>
+      </c>
+      <c r="F9" s="11">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="12">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11">
+        <v>96</v>
+      </c>
+      <c r="C10" s="11">
+        <v>96</v>
+      </c>
+      <c r="D10" s="11">
+        <v>90</v>
+      </c>
+      <c r="E10" s="11">
+        <v>59</v>
+      </c>
+      <c r="F10" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="12">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11">
+        <v>48</v>
+      </c>
+      <c r="C11" s="11">
+        <v>98</v>
+      </c>
+      <c r="D11" s="11">
+        <v>58</v>
+      </c>
+      <c r="E11" s="11">
+        <v>79</v>
+      </c>
+      <c r="F11" s="11">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="11">
+        <v>49</v>
+      </c>
+      <c r="C12" s="11">
+        <v>85</v>
+      </c>
+      <c r="D12" s="11">
+        <v>59</v>
+      </c>
+      <c r="E12" s="11">
+        <v>96</v>
+      </c>
+      <c r="F12" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="12">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11">
+        <v>71</v>
+      </c>
+      <c r="C13" s="11">
+        <v>15</v>
+      </c>
+      <c r="D13" s="11">
+        <v>72</v>
+      </c>
+      <c r="E13" s="11">
+        <v>95</v>
+      </c>
+      <c r="F13" s="11">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="12">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11">
+        <v>95</v>
+      </c>
+      <c r="C14" s="11">
+        <v>45</v>
+      </c>
+      <c r="D14" s="11">
+        <v>87</v>
+      </c>
+      <c r="E14" s="11">
+        <v>98</v>
+      </c>
+      <c r="F14" s="11">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="12">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11">
+        <v>37</v>
+      </c>
+      <c r="C15" s="11">
+        <v>19</v>
+      </c>
+      <c r="D15" s="11">
+        <v>79</v>
+      </c>
+      <c r="E15" s="11">
+        <v>28</v>
+      </c>
+      <c r="F15" s="11">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="12">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11">
+        <v>83</v>
+      </c>
+      <c r="C16" s="11">
+        <v>99</v>
+      </c>
+      <c r="D16" s="11">
+        <v>91</v>
+      </c>
+      <c r="E16" s="11">
+        <v>12</v>
+      </c>
+      <c r="F16" s="11">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="12">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11">
+        <v>85</v>
+      </c>
+      <c r="C17" s="11">
+        <v>95</v>
+      </c>
+      <c r="D17" s="11">
+        <v>46</v>
+      </c>
+      <c r="E17" s="11">
+        <v>37</v>
+      </c>
+      <c r="F17" s="11">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="12">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11">
+        <v>93</v>
+      </c>
+      <c r="C18" s="11">
+        <v>100</v>
+      </c>
+      <c r="D18" s="11">
+        <v>66</v>
+      </c>
+      <c r="E18" s="11">
+        <v>76</v>
+      </c>
+      <c r="F18" s="11">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="12">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11">
+        <v>69</v>
+      </c>
+      <c r="C19" s="11">
+        <v>98</v>
+      </c>
+      <c r="D19" s="11">
+        <v>53</v>
+      </c>
+      <c r="E19" s="11">
+        <v>94</v>
+      </c>
+      <c r="F19" s="11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="12">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11">
+        <v>86</v>
+      </c>
+      <c r="C20" s="11">
+        <v>33</v>
+      </c>
+      <c r="D20" s="11">
+        <v>71</v>
+      </c>
+      <c r="E20" s="11">
+        <v>84</v>
+      </c>
+      <c r="F20" s="11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="12">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11">
+        <v>66</v>
+      </c>
+      <c r="C21" s="11">
+        <v>70</v>
+      </c>
+      <c r="D21" s="11">
+        <v>99</v>
+      </c>
+      <c r="E21" s="11">
+        <v>86</v>
+      </c>
+      <c r="F21" s="11">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="12">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11">
+        <v>84</v>
+      </c>
+      <c r="C22" s="11">
+        <v>94</v>
+      </c>
+      <c r="D22" s="11">
+        <v>80</v>
+      </c>
+      <c r="E22" s="11">
+        <v>50</v>
+      </c>
+      <c r="F22" s="11">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="12">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11">
+        <v>89</v>
+      </c>
+      <c r="C23" s="11">
+        <v>50</v>
+      </c>
+      <c r="D23" s="11">
+        <v>70</v>
+      </c>
+      <c r="E23" s="11">
+        <v>90</v>
+      </c>
+      <c r="F23" s="11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="12">
+        <v>23</v>
+      </c>
+      <c r="B24" s="11">
+        <v>73</v>
+      </c>
+      <c r="C24" s="11">
+        <v>88</v>
+      </c>
+      <c r="D24" s="11">
+        <v>96</v>
+      </c>
+      <c r="E24" s="11">
+        <v>94</v>
+      </c>
+      <c r="F24" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="12">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11">
+        <v>46</v>
+      </c>
+      <c r="C25" s="11">
+        <v>32</v>
+      </c>
+      <c r="D25" s="11">
+        <v>97</v>
+      </c>
+      <c r="E25" s="11">
+        <v>90</v>
+      </c>
+      <c r="F25" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="12">
+        <v>25</v>
+      </c>
+      <c r="B26" s="11">
+        <v>80</v>
+      </c>
+      <c r="C26" s="11">
+        <v>61</v>
+      </c>
+      <c r="D26" s="11">
+        <v>81</v>
+      </c>
+      <c r="E26" s="11">
+        <v>66</v>
+      </c>
+      <c r="F26" s="11">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="12">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11">
+        <v>61</v>
+      </c>
+      <c r="C27" s="11">
+        <v>62</v>
+      </c>
+      <c r="D27" s="11">
+        <v>45</v>
+      </c>
+      <c r="E27" s="11">
+        <v>78</v>
+      </c>
+      <c r="F27" s="11">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A28" s="12">
+        <v>27</v>
+      </c>
+      <c r="B28" s="11">
+        <v>99</v>
+      </c>
+      <c r="C28" s="11">
+        <v>75</v>
+      </c>
+      <c r="D28" s="11">
+        <v>90</v>
+      </c>
+      <c r="E28" s="11">
+        <v>95</v>
+      </c>
+      <c r="F28" s="11">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29" s="12">
+        <v>28</v>
+      </c>
+      <c r="B29" s="11">
+        <v>90</v>
+      </c>
+      <c r="C29" s="11">
+        <v>89</v>
+      </c>
+      <c r="D29" s="11">
+        <v>89</v>
+      </c>
+      <c r="E29" s="11">
+        <v>35</v>
+      </c>
+      <c r="F29" s="11">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="12">
+        <v>29</v>
+      </c>
+      <c r="B30" s="11">
+        <v>91</v>
+      </c>
+      <c r="C30" s="11">
+        <v>68</v>
+      </c>
+      <c r="D30" s="11">
+        <v>97</v>
+      </c>
+      <c r="E30" s="11">
+        <v>42</v>
+      </c>
+      <c r="F30" s="11">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31" s="12">
+        <v>30</v>
+      </c>
+      <c r="B31" s="11">
+        <v>45</v>
+      </c>
+      <c r="C31" s="11">
+        <v>96</v>
+      </c>
+      <c r="D31" s="11">
+        <v>53</v>
+      </c>
+      <c r="E31" s="11">
+        <v>57</v>
+      </c>
+      <c r="F31" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="12">
+        <v>31</v>
+      </c>
+      <c r="B32" s="11">
+        <v>22</v>
+      </c>
+      <c r="C32" s="11">
+        <v>72</v>
+      </c>
+      <c r="D32" s="11">
+        <v>89</v>
+      </c>
+      <c r="E32" s="11">
+        <v>80</v>
+      </c>
+      <c r="F32" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="12">
+        <v>32</v>
+      </c>
+      <c r="B33" s="11">
+        <v>82</v>
+      </c>
+      <c r="C33" s="11">
+        <v>79</v>
+      </c>
+      <c r="D33" s="11">
+        <v>66</v>
+      </c>
+      <c r="E33" s="11">
+        <v>91</v>
+      </c>
+      <c r="F33" s="11">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A34" s="12">
+        <v>33</v>
+      </c>
+      <c r="B34" s="11">
+        <v>93</v>
+      </c>
+      <c r="C34" s="11">
+        <v>94</v>
+      </c>
+      <c r="D34" s="11">
+        <v>92</v>
+      </c>
+      <c r="E34" s="11">
+        <v>83</v>
+      </c>
+      <c r="F34" s="11">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A35" s="12">
+        <v>34</v>
+      </c>
+      <c r="B35" s="11">
+        <v>43</v>
+      </c>
+      <c r="C35" s="11">
+        <v>100</v>
+      </c>
+      <c r="D35" s="11">
+        <v>68</v>
+      </c>
+      <c r="E35" s="11">
+        <v>81</v>
+      </c>
+      <c r="F35" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A36" s="12">
+        <v>35</v>
+      </c>
+      <c r="B36" s="11">
+        <v>68</v>
+      </c>
+      <c r="C36" s="11">
+        <v>46</v>
+      </c>
+      <c r="D36" s="11">
+        <v>99</v>
+      </c>
+      <c r="E36" s="11">
+        <v>67</v>
+      </c>
+      <c r="F36" s="11">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="12">
+        <v>36</v>
+      </c>
+      <c r="B37" s="11">
+        <v>73</v>
+      </c>
+      <c r="C37" s="11">
+        <v>90</v>
+      </c>
+      <c r="D37" s="11">
+        <v>72</v>
+      </c>
+      <c r="E37" s="11">
+        <v>77</v>
+      </c>
+      <c r="F37" s="11">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="12">
+        <v>37</v>
+      </c>
+      <c r="B38" s="11">
+        <v>60</v>
+      </c>
+      <c r="C38" s="11">
+        <v>79</v>
+      </c>
+      <c r="D38" s="11">
+        <v>99</v>
+      </c>
+      <c r="E38" s="11">
+        <v>86</v>
+      </c>
+      <c r="F38" s="11">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="12">
+        <v>38</v>
+      </c>
+      <c r="B39" s="11">
+        <v>46</v>
+      </c>
+      <c r="C39" s="11">
+        <v>56</v>
+      </c>
+      <c r="D39" s="11">
+        <v>65</v>
+      </c>
+      <c r="E39" s="11">
+        <v>73</v>
+      </c>
+      <c r="F39" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A40" s="12">
+        <v>39</v>
+      </c>
+      <c r="B40" s="11">
+        <v>56</v>
+      </c>
+      <c r="C40" s="11">
+        <v>51</v>
+      </c>
+      <c r="D40" s="11">
+        <v>98</v>
+      </c>
+      <c r="E40" s="11">
+        <v>69</v>
+      </c>
+      <c r="F40" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41" s="12">
+        <v>40</v>
+      </c>
+      <c r="B41" s="11">
+        <v>95</v>
+      </c>
+      <c r="C41" s="11">
+        <v>78</v>
+      </c>
+      <c r="D41" s="11">
+        <v>84</v>
+      </c>
+      <c r="E41" s="11">
+        <v>90</v>
+      </c>
+      <c r="F41" s="11">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="12">
+        <v>41</v>
+      </c>
+      <c r="B42" s="11">
+        <v>70</v>
+      </c>
+      <c r="C42" s="11">
+        <v>57</v>
+      </c>
+      <c r="D42" s="11">
+        <v>98</v>
+      </c>
+      <c r="E42" s="11">
+        <v>87</v>
+      </c>
+      <c r="F42" s="11">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A43" s="12">
+        <v>42</v>
+      </c>
+      <c r="B43" s="11">
+        <v>67</v>
+      </c>
+      <c r="C43" s="11">
+        <v>26</v>
+      </c>
+      <c r="D43" s="11">
+        <v>94</v>
+      </c>
+      <c r="E43" s="11">
+        <v>93</v>
+      </c>
+      <c r="F43" s="11">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A44" s="12">
+        <v>43</v>
+      </c>
+      <c r="B44" s="11">
+        <v>38</v>
+      </c>
+      <c r="C44" s="11">
+        <v>91</v>
+      </c>
+      <c r="D44" s="11">
+        <v>58</v>
+      </c>
+      <c r="E44" s="11">
+        <v>86</v>
+      </c>
+      <c r="F44" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A45" s="12">
+        <v>44</v>
+      </c>
+      <c r="B45" s="11">
+        <v>52</v>
+      </c>
+      <c r="C45" s="11">
+        <v>83</v>
+      </c>
+      <c r="D45" s="11">
+        <v>93</v>
+      </c>
+      <c r="E45" s="11">
+        <v>64</v>
+      </c>
+      <c r="F45" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A46" s="12">
+        <v>45</v>
+      </c>
+      <c r="B46" s="11">
+        <v>62</v>
+      </c>
+      <c r="C46" s="11">
+        <v>66</v>
+      </c>
+      <c r="D46" s="11">
+        <v>71</v>
+      </c>
+      <c r="E46" s="11">
+        <v>84</v>
+      </c>
+      <c r="F46" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A47" s="12">
+        <v>46</v>
+      </c>
+      <c r="B47" s="11">
+        <v>99</v>
+      </c>
+      <c r="C47" s="11">
+        <v>19</v>
+      </c>
+      <c r="D47" s="11">
+        <v>81</v>
+      </c>
+      <c r="E47" s="11">
+        <v>75</v>
+      </c>
+      <c r="F47" s="11">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A48" s="12">
+        <v>47</v>
+      </c>
+      <c r="B48" s="11">
+        <v>53</v>
+      </c>
+      <c r="C48" s="11">
+        <v>90</v>
+      </c>
+      <c r="D48" s="11">
+        <v>86</v>
+      </c>
+      <c r="E48" s="11">
+        <v>92</v>
+      </c>
+      <c r="F48" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A49" s="12">
+        <v>48</v>
+      </c>
+      <c r="B49" s="11">
+        <v>82</v>
+      </c>
+      <c r="C49" s="11">
+        <v>98</v>
+      </c>
+      <c r="D49" s="11">
+        <v>89</v>
+      </c>
+      <c r="E49" s="11">
+        <v>66</v>
+      </c>
+      <c r="F49" s="11">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A50" s="12">
+        <v>49</v>
+      </c>
+      <c r="B50" s="11">
+        <v>68</v>
+      </c>
+      <c r="C50" s="11">
+        <v>97</v>
+      </c>
+      <c r="D50" s="11">
+        <v>40</v>
+      </c>
+      <c r="E50" s="11">
+        <v>89</v>
+      </c>
+      <c r="F50" s="11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A51" s="12">
+        <v>50</v>
+      </c>
+      <c r="B51" s="11">
+        <v>47</v>
+      </c>
+      <c r="C51" s="11">
+        <v>57</v>
+      </c>
+      <c r="D51" s="11">
+        <v>84</v>
+      </c>
+      <c r="E51" s="11">
+        <v>62</v>
+      </c>
+      <c r="F51" s="11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A52" s="12">
+        <v>51</v>
+      </c>
+      <c r="B52" s="11">
+        <v>80</v>
+      </c>
+      <c r="C52" s="11">
+        <v>89</v>
+      </c>
+      <c r="D52" s="11">
+        <v>82</v>
+      </c>
+      <c r="E52" s="11">
+        <v>88</v>
+      </c>
+      <c r="F52" s="11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A53" s="12">
+        <v>52</v>
+      </c>
+      <c r="B53" s="11">
+        <v>60</v>
+      </c>
+      <c r="C53" s="11">
+        <v>70</v>
+      </c>
+      <c r="D53" s="11">
+        <v>76</v>
+      </c>
+      <c r="E53" s="11">
+        <v>36</v>
+      </c>
+      <c r="F53" s="11">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A54" s="12">
+        <v>53</v>
+      </c>
+      <c r="B54" s="11">
+        <v>49</v>
+      </c>
+      <c r="C54" s="11">
+        <v>92</v>
+      </c>
+      <c r="D54" s="11">
+        <v>43</v>
+      </c>
+      <c r="E54" s="11">
+        <v>81</v>
+      </c>
+      <c r="F54" s="11">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A55" s="12">
+        <v>54</v>
+      </c>
+      <c r="B55" s="11">
+        <v>60</v>
+      </c>
+      <c r="C55" s="11">
+        <v>25</v>
+      </c>
+      <c r="D55" s="11">
+        <v>56</v>
+      </c>
+      <c r="E55" s="11">
+        <v>100</v>
+      </c>
+      <c r="F55" s="11">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A56" s="12">
+        <v>55</v>
+      </c>
+      <c r="B56" s="11">
+        <v>50</v>
+      </c>
+      <c r="C56" s="11">
+        <v>63</v>
+      </c>
+      <c r="D56" s="11">
+        <v>97</v>
+      </c>
+      <c r="E56" s="11">
+        <v>98</v>
+      </c>
+      <c r="F56" s="11">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A57" s="12">
+        <v>56</v>
+      </c>
+      <c r="B57" s="11">
+        <v>69</v>
+      </c>
+      <c r="C57" s="11">
+        <v>91</v>
+      </c>
+      <c r="D57" s="11">
+        <v>40</v>
+      </c>
+      <c r="E57" s="11">
+        <v>95</v>
+      </c>
+      <c r="F57" s="11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A58" s="12">
+        <v>57</v>
+      </c>
+      <c r="B58" s="11">
+        <v>72</v>
+      </c>
+      <c r="C58" s="11">
+        <v>91</v>
+      </c>
+      <c r="D58" s="11">
+        <v>60</v>
+      </c>
+      <c r="E58" s="11">
+        <v>81</v>
+      </c>
+      <c r="F58" s="11">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A59" s="12">
+        <v>58</v>
+      </c>
+      <c r="B59" s="11">
+        <v>87</v>
+      </c>
+      <c r="C59" s="11">
+        <v>92</v>
+      </c>
+      <c r="D59" s="11">
+        <v>78</v>
+      </c>
+      <c r="E59" s="11">
+        <v>72</v>
+      </c>
+      <c r="F59" s="11">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A60" s="12">
+        <v>59</v>
+      </c>
+      <c r="B60" s="11">
+        <v>47</v>
+      </c>
+      <c r="C60" s="11">
+        <v>88</v>
+      </c>
+      <c r="D60" s="11">
+        <v>65</v>
+      </c>
+      <c r="E60" s="11">
+        <v>100</v>
+      </c>
+      <c r="F60" s="11">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A61" s="12">
+        <v>60</v>
+      </c>
+      <c r="B61" s="11">
+        <v>50</v>
+      </c>
+      <c r="C61" s="11">
+        <v>64</v>
+      </c>
+      <c r="D61" s="11">
+        <v>94</v>
+      </c>
+      <c r="E61" s="11">
+        <v>67</v>
+      </c>
+      <c r="F61" s="11">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A62" s="12">
+        <v>61</v>
+      </c>
+      <c r="B62" s="11">
+        <v>64</v>
+      </c>
+      <c r="C62" s="11">
+        <v>91</v>
+      </c>
+      <c r="D62" s="11">
+        <v>86</v>
+      </c>
+      <c r="E62" s="11">
+        <v>60</v>
+      </c>
+      <c r="F62" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A63" s="12">
+        <v>62</v>
+      </c>
+      <c r="B63" s="11">
+        <v>97</v>
+      </c>
+      <c r="C63" s="11">
+        <v>49</v>
+      </c>
+      <c r="D63" s="11">
+        <v>24</v>
+      </c>
+      <c r="E63" s="11">
+        <v>73</v>
+      </c>
+      <c r="F63" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A64" s="12">
+        <v>63</v>
+      </c>
+      <c r="B64" s="11">
+        <v>93</v>
+      </c>
+      <c r="C64" s="11">
+        <v>51</v>
+      </c>
+      <c r="D64" s="11">
+        <v>72</v>
+      </c>
+      <c r="E64" s="11">
+        <v>74</v>
+      </c>
+      <c r="F64" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="12">
+        <v>64</v>
+      </c>
+      <c r="B65" s="11">
+        <v>71</v>
+      </c>
+      <c r="C65" s="11">
+        <v>76</v>
+      </c>
+      <c r="D65" s="11">
+        <v>52</v>
+      </c>
+      <c r="E65" s="11">
+        <v>81</v>
+      </c>
+      <c r="F65" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A66" s="12">
+        <v>65</v>
+      </c>
+      <c r="B66" s="11">
+        <v>90</v>
+      </c>
+      <c r="C66" s="11">
+        <v>88</v>
+      </c>
+      <c r="D66" s="11">
+        <v>88</v>
+      </c>
+      <c r="E66" s="11">
+        <v>100</v>
+      </c>
+      <c r="F66" s="11">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="12">
+        <v>66</v>
+      </c>
+      <c r="B67" s="11">
+        <v>61</v>
+      </c>
+      <c r="C67" s="11">
+        <v>93</v>
+      </c>
+      <c r="D67" s="11">
+        <v>82</v>
+      </c>
+      <c r="E67" s="11">
+        <v>97</v>
+      </c>
+      <c r="F67" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="12">
+        <v>67</v>
+      </c>
+      <c r="B68" s="11">
+        <v>33</v>
+      </c>
+      <c r="C68" s="11">
+        <v>26</v>
+      </c>
+      <c r="D68" s="11">
+        <v>71</v>
+      </c>
+      <c r="E68" s="11">
+        <v>77</v>
+      </c>
+      <c r="F68" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A69" s="12">
+        <v>68</v>
+      </c>
+      <c r="B69" s="11">
+        <v>92</v>
+      </c>
+      <c r="C69" s="11">
+        <v>6666</v>
+      </c>
+      <c r="D69" s="11">
+        <v>30</v>
+      </c>
+      <c r="E69" s="11">
+        <v>96</v>
+      </c>
+      <c r="F69" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A70" s="12">
+        <v>69</v>
+      </c>
+      <c r="B70" s="11">
+        <v>81</v>
+      </c>
+      <c r="C70" s="11">
+        <v>58</v>
+      </c>
+      <c r="D70" s="11">
+        <v>83</v>
+      </c>
+      <c r="E70" s="11">
+        <v>21</v>
+      </c>
+      <c r="F70" s="11">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A71" s="12">
+        <v>70</v>
+      </c>
+      <c r="B71" s="11">
+        <v>41</v>
+      </c>
+      <c r="C71" s="11">
+        <v>79</v>
+      </c>
+      <c r="D71" s="11">
+        <v>82</v>
+      </c>
+      <c r="E71" s="11">
+        <v>58</v>
+      </c>
+      <c r="F71" s="11">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A72" s="12">
+        <v>71</v>
+      </c>
+      <c r="B72" s="11">
+        <v>87</v>
+      </c>
+      <c r="C72" s="11">
+        <v>80</v>
+      </c>
+      <c r="D72" s="11">
+        <v>80</v>
+      </c>
+      <c r="E72" s="11">
+        <v>75</v>
+      </c>
+      <c r="F72" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A73" s="12">
+        <v>72</v>
+      </c>
+      <c r="B73" s="11">
+        <v>57</v>
+      </c>
+      <c r="C73" s="11">
+        <v>89</v>
+      </c>
+      <c r="D73" s="11">
+        <v>89</v>
+      </c>
+      <c r="E73" s="11">
+        <v>997</v>
+      </c>
+      <c r="F73" s="11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A74" s="12">
+        <v>73</v>
+      </c>
+      <c r="B74" s="11">
+        <v>92</v>
+      </c>
+      <c r="C74" s="11">
+        <v>46</v>
+      </c>
+      <c r="D74" s="11">
+        <v>74</v>
+      </c>
+      <c r="E74" s="11">
+        <v>97</v>
+      </c>
+      <c r="F74" s="11">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A75" s="12">
+        <v>74</v>
+      </c>
+      <c r="B75" s="11">
+        <v>84</v>
+      </c>
+      <c r="C75" s="11">
+        <v>64</v>
+      </c>
+      <c r="D75" s="11">
+        <v>99</v>
+      </c>
+      <c r="E75" s="11">
+        <v>97</v>
+      </c>
+      <c r="F75" s="11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A76" s="12">
+        <v>75</v>
+      </c>
+      <c r="B76" s="11">
+        <v>87</v>
+      </c>
+      <c r="C76" s="11">
+        <v>99</v>
+      </c>
+      <c r="D76" s="11">
+        <v>86</v>
+      </c>
+      <c r="E76" s="11">
+        <v>97</v>
+      </c>
+      <c r="F76" s="11">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A77" s="12">
+        <v>76</v>
+      </c>
+      <c r="B77" s="11">
+        <v>37</v>
+      </c>
+      <c r="C77" s="11">
+        <v>97</v>
+      </c>
+      <c r="D77" s="11">
+        <v>59</v>
+      </c>
+      <c r="E77" s="11">
+        <v>64</v>
+      </c>
+      <c r="F77" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A78" s="12">
+        <v>77</v>
+      </c>
+      <c r="B78" s="11">
+        <v>86</v>
+      </c>
+      <c r="C78" s="11">
+        <v>100</v>
+      </c>
+      <c r="D78" s="11">
+        <v>89</v>
+      </c>
+      <c r="E78" s="11">
+        <v>100</v>
+      </c>
+      <c r="F78" s="11">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A79" s="12">
+        <v>78</v>
+      </c>
+      <c r="B79" s="11">
+        <v>96</v>
+      </c>
+      <c r="C79" s="11">
+        <v>72</v>
+      </c>
+      <c r="D79" s="11">
+        <v>34</v>
+      </c>
+      <c r="E79" s="11">
+        <v>97</v>
+      </c>
+      <c r="F79" s="11">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A80" s="12">
+        <v>79</v>
+      </c>
+      <c r="B80" s="11">
+        <v>81</v>
+      </c>
+      <c r="C80" s="11">
+        <v>34</v>
+      </c>
+      <c r="D80" s="11">
+        <v>98</v>
+      </c>
+      <c r="E80" s="11">
+        <v>54</v>
+      </c>
+      <c r="F80" s="11">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A81" s="12">
+        <v>80</v>
+      </c>
+      <c r="B81" s="11">
+        <v>94</v>
+      </c>
+      <c r="C81" s="11">
+        <v>94</v>
+      </c>
+      <c r="D81" s="11">
+        <v>96</v>
+      </c>
+      <c r="E81" s="11">
+        <v>62</v>
+      </c>
+      <c r="F81" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A82" s="12">
+        <v>81</v>
+      </c>
+      <c r="B82" s="11">
+        <v>73</v>
+      </c>
+      <c r="C82" s="11">
+        <v>56</v>
+      </c>
+      <c r="D82" s="11">
+        <v>70</v>
+      </c>
+      <c r="E82" s="11">
+        <v>17</v>
+      </c>
+      <c r="F82" s="11">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A83" s="12">
+        <v>82</v>
+      </c>
+      <c r="B83" s="11">
+        <v>69</v>
+      </c>
+      <c r="C83" s="11">
+        <v>94</v>
+      </c>
+      <c r="D83" s="11">
+        <v>73</v>
+      </c>
+      <c r="E83" s="11">
+        <v>92</v>
+      </c>
+      <c r="F83" s="11">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A84" s="12">
+        <v>83</v>
+      </c>
+      <c r="B84" s="11">
+        <v>87</v>
+      </c>
+      <c r="C84" s="11">
+        <v>73</v>
+      </c>
+      <c r="D84" s="11">
+        <v>98</v>
+      </c>
+      <c r="E84" s="11">
+        <v>87</v>
+      </c>
+      <c r="F84" s="11">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A85" s="12">
+        <v>84</v>
+      </c>
+      <c r="B85" s="11">
+        <v>83</v>
+      </c>
+      <c r="C85" s="11">
+        <v>33</v>
+      </c>
+      <c r="D85" s="11">
+        <v>32</v>
+      </c>
+      <c r="E85" s="11">
+        <v>49</v>
+      </c>
+      <c r="F85" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A86" s="12">
+        <v>85</v>
+      </c>
+      <c r="B86" s="11">
+        <v>84</v>
+      </c>
+      <c r="C86" s="11">
+        <v>83</v>
+      </c>
+      <c r="D86" s="11">
+        <v>100</v>
+      </c>
+      <c r="E86" s="11">
+        <v>0.67</v>
+      </c>
+      <c r="F86" s="11">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A87" s="12">
+        <v>86</v>
+      </c>
+      <c r="B87" s="11">
+        <v>100</v>
+      </c>
+      <c r="C87" s="11">
+        <v>87</v>
+      </c>
+      <c r="D87" s="11">
+        <v>36</v>
+      </c>
+      <c r="E87" s="11">
+        <v>79</v>
+      </c>
+      <c r="F87" s="11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A88" s="12">
+        <v>87</v>
+      </c>
+      <c r="B88" s="11">
+        <v>55</v>
+      </c>
+      <c r="C88" s="11">
+        <v>86</v>
+      </c>
+      <c r="D88" s="11">
+        <v>85</v>
+      </c>
+      <c r="E88" s="11">
+        <v>95</v>
+      </c>
+      <c r="F88" s="11">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A89" s="12">
+        <v>88</v>
+      </c>
+      <c r="B89" s="11">
+        <v>71</v>
+      </c>
+      <c r="C89" s="11">
+        <v>98</v>
+      </c>
+      <c r="D89" s="11">
+        <v>36</v>
+      </c>
+      <c r="E89" s="11">
+        <v>94</v>
+      </c>
+      <c r="F89" s="11">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A90" s="12">
+        <v>89</v>
+      </c>
+      <c r="B90" s="11">
+        <v>97</v>
+      </c>
+      <c r="C90" s="11">
+        <v>54</v>
+      </c>
+      <c r="D90" s="11">
+        <v>73</v>
+      </c>
+      <c r="E90" s="11">
+        <v>58</v>
+      </c>
+      <c r="F90" s="11">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A91" s="12">
+        <v>90</v>
+      </c>
+      <c r="B91" s="11">
+        <v>8.4</v>
+      </c>
+      <c r="C91" s="11">
+        <v>88</v>
+      </c>
+      <c r="D91" s="11">
+        <v>93</v>
+      </c>
+      <c r="E91" s="11">
+        <v>65</v>
+      </c>
+      <c r="F91" s="11">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A92" s="12">
+        <v>91</v>
+      </c>
+      <c r="B92" s="11">
+        <v>93</v>
+      </c>
+      <c r="C92" s="11">
+        <v>80</v>
+      </c>
+      <c r="D92" s="11">
+        <v>19</v>
+      </c>
+      <c r="E92" s="11">
+        <v>96</v>
+      </c>
+      <c r="F92" s="11">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A93" s="12">
+        <v>92</v>
+      </c>
+      <c r="B93" s="11">
+        <v>48</v>
+      </c>
+      <c r="C93" s="11">
+        <v>86</v>
+      </c>
+      <c r="D93" s="11">
+        <v>83</v>
+      </c>
+      <c r="E93" s="11">
+        <v>92</v>
+      </c>
+      <c r="F93" s="11">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A94" s="12">
+        <v>93</v>
+      </c>
+      <c r="B94" s="11">
+        <v>64</v>
+      </c>
+      <c r="C94" s="11">
+        <v>87</v>
+      </c>
+      <c r="D94" s="11">
+        <v>35</v>
+      </c>
+      <c r="E94" s="11">
+        <v>41</v>
+      </c>
+      <c r="F94" s="11">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A95" s="12">
+        <v>94</v>
+      </c>
+      <c r="B95" s="11">
+        <v>76</v>
+      </c>
+      <c r="C95" s="11">
+        <v>100</v>
+      </c>
+      <c r="D95" s="11">
+        <v>83</v>
+      </c>
+      <c r="E95" s="11">
+        <v>70</v>
+      </c>
+      <c r="F95" s="11">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A96" s="12">
+        <v>95</v>
+      </c>
+      <c r="B96" s="11">
+        <v>69</v>
+      </c>
+      <c r="C96" s="11">
+        <v>44</v>
+      </c>
+      <c r="D96" s="11">
+        <v>90</v>
+      </c>
+      <c r="E96" s="11">
+        <v>79</v>
+      </c>
+      <c r="F96" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A97" s="12">
+        <v>96</v>
+      </c>
+      <c r="B97" s="11">
+        <v>94</v>
+      </c>
+      <c r="C97" s="11">
+        <v>77</v>
+      </c>
+      <c r="D97" s="11">
+        <v>41</v>
+      </c>
+      <c r="E97" s="11">
+        <v>94</v>
+      </c>
+      <c r="F97" s="11">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A98" s="12">
+        <v>97</v>
+      </c>
+      <c r="B98" s="11">
+        <v>63</v>
+      </c>
+      <c r="C98" s="11">
+        <v>91</v>
+      </c>
+      <c r="D98" s="11">
+        <v>82</v>
+      </c>
+      <c r="E98" s="11">
+        <v>63</v>
+      </c>
+      <c r="F98" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A99" s="12">
+        <v>98</v>
+      </c>
+      <c r="B99" s="11">
+        <v>72</v>
+      </c>
+      <c r="C99" s="11">
+        <v>20</v>
+      </c>
+      <c r="D99" s="11">
+        <v>97</v>
+      </c>
+      <c r="E99" s="11">
+        <v>59</v>
+      </c>
+      <c r="F99" s="11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A100" s="12">
+        <v>99</v>
+      </c>
+      <c r="B100" s="11">
+        <v>96</v>
+      </c>
+      <c r="C100" s="11">
+        <v>31</v>
+      </c>
+      <c r="D100" s="11">
+        <v>89</v>
+      </c>
+      <c r="E100" s="11">
+        <v>45</v>
+      </c>
+      <c r="F100" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A101" s="12">
+        <v>100</v>
+      </c>
+      <c r="B101" s="11">
+        <v>79</v>
+      </c>
+      <c r="C101" s="11">
+        <v>93</v>
+      </c>
+      <c r="D101" s="11">
+        <v>68</v>
+      </c>
+      <c r="E101" s="11">
+        <v>94</v>
+      </c>
+      <c r="F101" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A102" s="12">
+        <v>101</v>
+      </c>
+      <c r="B102" s="11">
+        <v>64</v>
+      </c>
+      <c r="C102" s="11">
+        <v>52</v>
+      </c>
+      <c r="D102" s="11">
+        <v>92</v>
+      </c>
+      <c r="E102" s="11">
+        <v>76</v>
+      </c>
+      <c r="F102" s="11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A103" s="12">
+        <v>102</v>
+      </c>
+      <c r="B103" s="11">
+        <v>99</v>
+      </c>
+      <c r="C103" s="11">
+        <v>97</v>
+      </c>
+      <c r="D103" s="11">
+        <v>86</v>
+      </c>
+      <c r="E103" s="11">
+        <v>100</v>
+      </c>
+      <c r="F103" s="11">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A104" s="12">
+        <v>103</v>
+      </c>
+      <c r="B104" s="11">
+        <v>49</v>
+      </c>
+      <c r="C104" s="11">
+        <v>86</v>
+      </c>
+      <c r="D104" s="11">
+        <v>77</v>
+      </c>
+      <c r="E104" s="11">
+        <v>48</v>
+      </c>
+      <c r="F104" s="11">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A105" s="12">
+        <v>104</v>
+      </c>
+      <c r="B105" s="11">
+        <v>70</v>
+      </c>
+      <c r="C105" s="11">
+        <v>69</v>
+      </c>
+      <c r="D105" s="11">
+        <v>42</v>
+      </c>
+      <c r="E105" s="11">
+        <v>74</v>
+      </c>
+      <c r="F105" s="11">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A106" s="12">
+        <v>105</v>
+      </c>
+      <c r="B106" s="11">
+        <v>96</v>
+      </c>
+      <c r="C106" s="11">
+        <v>98</v>
+      </c>
+      <c r="D106" s="11">
+        <v>98</v>
+      </c>
+      <c r="E106" s="11">
+        <v>42</v>
+      </c>
+      <c r="F106" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A107" s="12">
+        <v>106</v>
+      </c>
+      <c r="B107" s="11">
+        <v>86</v>
+      </c>
+      <c r="C107" s="11">
+        <v>93</v>
+      </c>
+      <c r="D107" s="11">
+        <v>99</v>
+      </c>
+      <c r="E107" s="11">
+        <v>92</v>
+      </c>
+      <c r="F107" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A108" s="12">
+        <v>107</v>
+      </c>
+      <c r="B108" s="11">
+        <v>97</v>
+      </c>
+      <c r="C108" s="11">
+        <v>87</v>
+      </c>
+      <c r="D108" s="11">
+        <v>85</v>
+      </c>
+      <c r="E108" s="11">
+        <v>71</v>
+      </c>
+      <c r="F108" s="11">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A109" s="12">
+        <v>108</v>
+      </c>
+      <c r="B109" s="11">
+        <v>60</v>
+      </c>
+      <c r="C109" s="11">
+        <v>64</v>
+      </c>
+      <c r="D109" s="11">
+        <v>78</v>
+      </c>
+      <c r="E109" s="11">
+        <v>86</v>
+      </c>
+      <c r="F109" s="11">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A110" s="12">
+        <v>109</v>
+      </c>
+      <c r="B110" s="11">
+        <v>90</v>
+      </c>
+      <c r="C110" s="11">
+        <v>96</v>
+      </c>
+      <c r="D110" s="11">
+        <v>95</v>
+      </c>
+      <c r="E110" s="11">
+        <v>97</v>
+      </c>
+      <c r="F110" s="11">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A111" s="12">
+        <v>110</v>
+      </c>
+      <c r="B111" s="11">
+        <v>86</v>
+      </c>
+      <c r="C111" s="11">
+        <v>76</v>
+      </c>
+      <c r="D111" s="11">
+        <v>100</v>
+      </c>
+      <c r="E111" s="11">
+        <v>69</v>
+      </c>
+      <c r="F111" s="11">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A112" s="12">
+        <v>111</v>
+      </c>
+      <c r="B112" s="11">
+        <v>30</v>
+      </c>
+      <c r="C112" s="11">
+        <v>59</v>
+      </c>
+      <c r="D112" s="11">
+        <v>91</v>
+      </c>
+      <c r="E112" s="11">
+        <v>92</v>
+      </c>
+      <c r="F112" s="11">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A113" s="12">
+        <v>112</v>
+      </c>
+      <c r="B113" s="11">
+        <v>75</v>
+      </c>
+      <c r="C113" s="11">
+        <v>74</v>
+      </c>
+      <c r="D113" s="11">
+        <v>93</v>
+      </c>
+      <c r="E113" s="11">
+        <v>85</v>
+      </c>
+      <c r="F113" s="11">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A114" s="12">
+        <v>113</v>
+      </c>
+      <c r="B114" s="11">
+        <v>84</v>
+      </c>
+      <c r="C114" s="11">
+        <v>17</v>
+      </c>
+      <c r="D114" s="11">
+        <v>82</v>
+      </c>
+      <c r="E114" s="11">
+        <v>45</v>
+      </c>
+      <c r="F114" s="11">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A115" s="12">
+        <v>114</v>
+      </c>
+      <c r="B115" s="11">
+        <v>69</v>
+      </c>
+      <c r="C115" s="11">
+        <v>100</v>
+      </c>
+      <c r="D115" s="11">
+        <v>61</v>
+      </c>
+      <c r="E115" s="11">
+        <v>82</v>
+      </c>
+      <c r="F115" s="11">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A116" s="12">
+        <v>115</v>
+      </c>
+      <c r="B116" s="11">
+        <v>82</v>
+      </c>
+      <c r="C116" s="11">
+        <v>31</v>
+      </c>
+      <c r="D116" s="11">
+        <v>87</v>
+      </c>
+      <c r="E116" s="11">
+        <v>95</v>
+      </c>
+      <c r="F116" s="11">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A117" s="12">
+        <v>116</v>
+      </c>
+      <c r="B117" s="11">
+        <v>96</v>
+      </c>
+      <c r="C117" s="11">
+        <v>27</v>
+      </c>
+      <c r="D117" s="11">
+        <v>49</v>
+      </c>
+      <c r="E117" s="11">
+        <v>76</v>
+      </c>
+      <c r="F117" s="11">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A118" s="12">
+        <v>117</v>
+      </c>
+      <c r="B118" s="11">
+        <v>77</v>
+      </c>
+      <c r="C118" s="11">
+        <v>75</v>
+      </c>
+      <c r="D118" s="11">
+        <v>75</v>
+      </c>
+      <c r="E118" s="11">
+        <v>76</v>
+      </c>
+      <c r="F118" s="11">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A119" s="12">
+        <v>118</v>
+      </c>
+      <c r="B119" s="11">
+        <v>56</v>
+      </c>
+      <c r="C119" s="11">
+        <v>64</v>
+      </c>
+      <c r="D119" s="11">
+        <v>96</v>
+      </c>
+      <c r="E119" s="11">
+        <v>92</v>
+      </c>
+      <c r="F119" s="11">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A120" s="12">
+        <v>119</v>
+      </c>
+      <c r="B120" s="11">
+        <v>70</v>
+      </c>
+      <c r="C120" s="11">
+        <v>78</v>
+      </c>
+      <c r="D120" s="11">
+        <v>98</v>
+      </c>
+      <c r="E120" s="11">
+        <v>67</v>
+      </c>
+      <c r="F120" s="11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A121" s="12">
+        <v>120</v>
+      </c>
+      <c r="B121" s="11">
+        <v>99</v>
+      </c>
+      <c r="C121" s="11">
+        <v>100</v>
+      </c>
+      <c r="D121" s="11">
+        <v>82</v>
+      </c>
+      <c r="E121" s="11">
+        <v>90</v>
+      </c>
+      <c r="F121" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A122" s="12">
+        <v>121</v>
+      </c>
+      <c r="B122" s="11">
+        <v>73</v>
+      </c>
+      <c r="C122" s="11">
+        <v>73</v>
+      </c>
+      <c r="D122" s="11">
+        <v>87</v>
+      </c>
+      <c r="E122" s="11">
+        <v>76</v>
+      </c>
+      <c r="F122" s="11">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A123" s="12">
+        <v>122</v>
+      </c>
+      <c r="B123" s="11">
+        <v>70</v>
+      </c>
+      <c r="C123" s="11">
+        <v>69</v>
+      </c>
+      <c r="D123" s="11">
+        <v>50</v>
+      </c>
+      <c r="E123" s="11">
+        <v>69</v>
+      </c>
+      <c r="F123" s="11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A124" s="12">
+        <v>123</v>
+      </c>
+      <c r="B124" s="11">
+        <v>65</v>
+      </c>
+      <c r="C124" s="11">
+        <v>34</v>
+      </c>
+      <c r="D124" s="11">
+        <v>93</v>
+      </c>
+      <c r="E124" s="11">
+        <v>85</v>
+      </c>
+      <c r="F124" s="11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A125" s="12">
+        <v>124</v>
+      </c>
+      <c r="B125" s="11">
+        <v>57</v>
+      </c>
+      <c r="C125" s="11">
+        <v>75</v>
+      </c>
+      <c r="D125" s="11">
+        <v>75</v>
+      </c>
+      <c r="E125" s="11">
+        <v>73</v>
+      </c>
+      <c r="F125" s="11">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A126" s="12">
+        <v>125</v>
+      </c>
+      <c r="B126" s="11">
+        <v>63</v>
+      </c>
+      <c r="C126" s="11">
+        <v>31</v>
+      </c>
+      <c r="D126" s="11">
+        <v>84</v>
+      </c>
+      <c r="E126" s="11">
+        <v>75</v>
+      </c>
+      <c r="F126" s="11">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A127" s="12">
+        <v>126</v>
+      </c>
+      <c r="B127" s="11">
+        <v>44</v>
+      </c>
+      <c r="C127" s="11">
+        <v>73</v>
+      </c>
+      <c r="D127" s="11">
+        <v>43</v>
+      </c>
+      <c r="E127" s="11">
+        <v>54</v>
+      </c>
+      <c r="F127" s="11">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A128" s="12">
+        <v>127</v>
+      </c>
+      <c r="B128" s="11">
+        <v>77</v>
+      </c>
+      <c r="C128" s="11">
+        <v>88</v>
+      </c>
+      <c r="D128" s="11">
+        <v>60</v>
+      </c>
+      <c r="E128" s="11">
+        <v>88</v>
+      </c>
+      <c r="F128" s="11">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A129" s="12">
+        <v>128</v>
+      </c>
+      <c r="B129" s="11">
+        <v>44</v>
+      </c>
+      <c r="C129" s="11">
+        <v>94</v>
+      </c>
+      <c r="D129" s="11">
+        <v>63</v>
+      </c>
+      <c r="E129" s="11">
+        <v>74</v>
+      </c>
+      <c r="F129" s="11">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A130" s="12">
+        <v>129</v>
+      </c>
+      <c r="B130" s="11">
+        <v>87</v>
+      </c>
+      <c r="C130" s="11">
+        <v>66</v>
+      </c>
+      <c r="D130" s="11">
+        <v>75</v>
+      </c>
+      <c r="E130" s="11">
+        <v>30</v>
+      </c>
+      <c r="F130" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A131" s="12">
+        <v>130</v>
+      </c>
+      <c r="B131" s="11">
+        <v>95</v>
+      </c>
+      <c r="C131" s="11">
+        <v>86</v>
+      </c>
+      <c r="D131" s="11">
+        <v>99</v>
+      </c>
+      <c r="E131" s="11">
+        <v>62</v>
+      </c>
+      <c r="F131" s="11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A132" s="12">
+        <v>131</v>
+      </c>
+      <c r="B132" s="11">
+        <v>100</v>
+      </c>
+      <c r="C132" s="11">
+        <v>92</v>
+      </c>
+      <c r="D132" s="11">
+        <v>57</v>
+      </c>
+      <c r="E132" s="11">
+        <v>91</v>
+      </c>
+      <c r="F132" s="11">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A133" s="12">
+        <v>132</v>
+      </c>
+      <c r="B133" s="11">
+        <v>85</v>
+      </c>
+      <c r="C133" s="11">
+        <v>90</v>
+      </c>
+      <c r="D133" s="11">
+        <v>82</v>
+      </c>
+      <c r="E133" s="11">
+        <v>41</v>
+      </c>
+      <c r="F133" s="11">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A134" s="12">
+        <v>133</v>
+      </c>
+      <c r="B134" s="11">
+        <v>75</v>
+      </c>
+      <c r="C134" s="11">
+        <v>96</v>
+      </c>
+      <c r="D134" s="11">
+        <v>72</v>
+      </c>
+      <c r="E134" s="11">
+        <v>72</v>
+      </c>
+      <c r="F134" s="11">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A135" s="12">
+        <v>134</v>
+      </c>
+      <c r="B135" s="11">
+        <v>93</v>
+      </c>
+      <c r="C135" s="11">
+        <v>82</v>
+      </c>
+      <c r="D135" s="11">
+        <v>58</v>
+      </c>
+      <c r="E135" s="11">
+        <v>57</v>
+      </c>
+      <c r="F135" s="11">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A136" s="12">
+        <v>135</v>
+      </c>
+      <c r="B136" s="11">
+        <v>76</v>
+      </c>
+      <c r="C136" s="11">
+        <v>64</v>
+      </c>
+      <c r="D136" s="11">
+        <v>67</v>
+      </c>
+      <c r="E136" s="11">
+        <v>32</v>
+      </c>
+      <c r="F136" s="11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A137" s="12">
+        <v>136</v>
+      </c>
+      <c r="B137" s="11">
+        <v>83</v>
+      </c>
+      <c r="C137" s="11">
+        <v>39</v>
+      </c>
+      <c r="D137" s="11">
+        <v>87</v>
+      </c>
+      <c r="E137" s="11">
+        <v>97</v>
+      </c>
+      <c r="F137" s="11">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A138" s="12">
+        <v>137</v>
+      </c>
+      <c r="B138" s="11">
+        <v>50</v>
+      </c>
+      <c r="C138" s="11">
+        <v>86</v>
+      </c>
+      <c r="D138" s="11">
+        <v>80</v>
+      </c>
+      <c r="E138" s="11">
+        <v>86</v>
+      </c>
+      <c r="F138" s="11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A139" s="12">
+        <v>138</v>
+      </c>
+      <c r="B139" s="11">
+        <v>87</v>
+      </c>
+      <c r="C139" s="11">
+        <v>85</v>
+      </c>
+      <c r="D139" s="11">
+        <v>35</v>
+      </c>
+      <c r="E139" s="11">
+        <v>100</v>
+      </c>
+      <c r="F139" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A140" s="12">
+        <v>139</v>
+      </c>
+      <c r="B140" s="11">
+        <v>84</v>
+      </c>
+      <c r="C140" s="11">
+        <v>79</v>
+      </c>
+      <c r="D140" s="11">
+        <v>97</v>
+      </c>
+      <c r="E140" s="11">
+        <v>77</v>
+      </c>
+      <c r="F140" s="11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A141" s="12">
+        <v>140</v>
+      </c>
+      <c r="B141" s="11">
+        <v>95</v>
+      </c>
+      <c r="C141" s="11">
+        <v>60</v>
+      </c>
+      <c r="D141" s="11">
+        <v>69</v>
+      </c>
+      <c r="E141" s="11">
+        <v>74</v>
+      </c>
+      <c r="F141" s="11">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A142" s="12">
+        <v>141</v>
+      </c>
+      <c r="B142" s="11">
+        <v>63</v>
+      </c>
+      <c r="C142" s="11">
+        <v>77</v>
+      </c>
+      <c r="D142" s="11">
+        <v>98</v>
+      </c>
+      <c r="E142" s="11">
+        <v>90</v>
+      </c>
+      <c r="F142" s="11">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A143" s="12">
+        <v>142</v>
+      </c>
+      <c r="B143" s="11">
+        <v>66</v>
+      </c>
+      <c r="C143" s="11">
+        <v>100</v>
+      </c>
+      <c r="D143" s="11">
+        <v>90</v>
+      </c>
+      <c r="E143" s="11">
+        <v>99</v>
+      </c>
+      <c r="F143" s="11">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A144" s="12">
+        <v>143</v>
+      </c>
+      <c r="B144" s="11">
+        <v>93</v>
+      </c>
+      <c r="C144" s="11">
+        <v>84</v>
+      </c>
+      <c r="D144" s="11">
+        <v>69</v>
+      </c>
+      <c r="E144" s="11">
+        <v>81</v>
+      </c>
+      <c r="F144" s="11">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A145" s="12">
+        <v>144</v>
+      </c>
+      <c r="B145" s="11">
+        <v>88</v>
+      </c>
+      <c r="C145" s="11">
+        <v>79</v>
+      </c>
+      <c r="D145" s="11">
+        <v>69</v>
+      </c>
+      <c r="E145" s="11">
+        <v>66</v>
+      </c>
+      <c r="F145" s="11">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A146" s="12">
+        <v>145</v>
+      </c>
+      <c r="B146" s="11">
+        <v>53</v>
+      </c>
+      <c r="C146" s="11">
+        <v>68</v>
+      </c>
+      <c r="D146" s="11">
+        <v>100</v>
+      </c>
+      <c r="E146" s="11">
+        <v>29</v>
+      </c>
+      <c r="F146" s="11">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A147" s="12">
+        <v>146</v>
+      </c>
+      <c r="B147" s="11">
+        <v>82</v>
+      </c>
+      <c r="C147" s="11">
+        <v>60</v>
+      </c>
+      <c r="D147" s="11">
+        <v>79</v>
+      </c>
+      <c r="E147" s="11">
+        <v>77</v>
+      </c>
+      <c r="F147" s="11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A148" s="12">
+        <v>147</v>
+      </c>
+      <c r="B148" s="11">
+        <v>65</v>
+      </c>
+      <c r="C148" s="11">
+        <v>89</v>
+      </c>
+      <c r="D148" s="11">
+        <v>90</v>
+      </c>
+      <c r="E148" s="11">
+        <v>96</v>
+      </c>
+      <c r="F148" s="11">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A149" s="12">
+        <v>148</v>
+      </c>
+      <c r="B149" s="11">
+        <v>87</v>
+      </c>
+      <c r="C149" s="11">
+        <v>96</v>
+      </c>
+      <c r="D149" s="11">
+        <v>96</v>
+      </c>
+      <c r="E149" s="11">
+        <v>69</v>
+      </c>
+      <c r="F149" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A150" s="12">
+        <v>149</v>
+      </c>
+      <c r="B150" s="11">
+        <v>62</v>
+      </c>
+      <c r="C150" s="11">
+        <v>80</v>
+      </c>
+      <c r="D150" s="11">
+        <v>84</v>
+      </c>
+      <c r="E150" s="11">
+        <v>74</v>
+      </c>
+      <c r="F150" s="11">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A151" s="12">
+        <v>150</v>
+      </c>
+      <c r="B151" s="11">
+        <v>72</v>
+      </c>
+      <c r="C151" s="11">
+        <v>84</v>
+      </c>
+      <c r="D151" s="11">
+        <v>100</v>
+      </c>
+      <c r="E151" s="11">
+        <v>71</v>
+      </c>
+      <c r="F151" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A152" s="12">
+        <v>151</v>
+      </c>
+      <c r="B152" s="11">
+        <v>45</v>
+      </c>
+      <c r="C152" s="11">
+        <v>83</v>
+      </c>
+      <c r="D152" s="11">
+        <v>70</v>
+      </c>
+      <c r="E152" s="11">
+        <v>91</v>
+      </c>
+      <c r="F152" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A153" s="12">
+        <v>152</v>
+      </c>
+      <c r="B153" s="11">
+        <v>68</v>
+      </c>
+      <c r="C153" s="11">
+        <v>94</v>
+      </c>
+      <c r="D153" s="11">
+        <v>67</v>
+      </c>
+      <c r="E153" s="11">
+        <v>99</v>
+      </c>
+      <c r="F153" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A154" s="12">
+        <v>153</v>
+      </c>
+      <c r="B154" s="11">
+        <v>82</v>
+      </c>
+      <c r="C154" s="11">
+        <v>91</v>
+      </c>
+      <c r="D154" s="11">
+        <v>88</v>
+      </c>
+      <c r="E154" s="11">
+        <v>97</v>
+      </c>
+      <c r="F154" s="11">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A155" s="12">
+        <v>154</v>
+      </c>
+      <c r="B155" s="11">
+        <v>100</v>
+      </c>
+      <c r="C155" s="11">
+        <v>71</v>
+      </c>
+      <c r="D155" s="11">
+        <v>66</v>
+      </c>
+      <c r="E155" s="11">
+        <v>29</v>
+      </c>
+      <c r="F155" s="11">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A156" s="12">
+        <v>155</v>
+      </c>
+      <c r="B156" s="11">
+        <v>93</v>
+      </c>
+      <c r="C156" s="11">
+        <v>88</v>
+      </c>
+      <c r="D156" s="11">
+        <v>92</v>
+      </c>
+      <c r="E156" s="11">
+        <v>31</v>
+      </c>
+      <c r="F156" s="11">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A157" s="12">
+        <v>156</v>
+      </c>
+      <c r="B157" s="11">
+        <v>53</v>
+      </c>
+      <c r="C157" s="11">
+        <v>36</v>
+      </c>
+      <c r="D157" s="11">
+        <v>86</v>
+      </c>
+      <c r="E157" s="11">
+        <v>98</v>
+      </c>
+      <c r="F157" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A158" s="12">
+        <v>157</v>
+      </c>
+      <c r="B158" s="11">
+        <v>48</v>
+      </c>
+      <c r="C158" s="11"/>
+      <c r="D158" s="11">
+        <v>85</v>
+      </c>
+      <c r="E158" s="11">
+        <v>32</v>
+      </c>
+      <c r="F158" s="11">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A159" s="12">
+        <v>158</v>
+      </c>
+      <c r="B159" s="11">
+        <v>89</v>
+      </c>
+      <c r="C159" s="11">
+        <v>93</v>
+      </c>
+      <c r="D159" s="11">
+        <v>96</v>
+      </c>
+      <c r="E159" s="11">
+        <v>45</v>
+      </c>
+      <c r="F159" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A160" s="12">
+        <v>159</v>
+      </c>
+      <c r="B160" s="11">
+        <v>84</v>
+      </c>
+      <c r="C160" s="11">
+        <v>67</v>
+      </c>
+      <c r="D160" s="11">
+        <v>99</v>
+      </c>
+      <c r="E160" s="11">
+        <v>97</v>
+      </c>
+      <c r="F160" s="11">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A161" s="12">
+        <v>160</v>
+      </c>
+      <c r="B161" s="11">
+        <v>98</v>
+      </c>
+      <c r="C161" s="11">
+        <v>100</v>
+      </c>
+      <c r="D161" s="11">
+        <v>90</v>
+      </c>
+      <c r="E161" s="11">
+        <v>99</v>
+      </c>
+      <c r="F161" s="11">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A162" s="12">
+        <v>161</v>
+      </c>
+      <c r="B162" s="11">
+        <v>100</v>
+      </c>
+      <c r="C162" s="11">
+        <v>83</v>
+      </c>
+      <c r="D162" s="11">
+        <v>92</v>
+      </c>
+      <c r="E162" s="11">
+        <v>82</v>
+      </c>
+      <c r="F162" s="11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A163" s="12">
+        <v>162</v>
+      </c>
+      <c r="B163" s="11">
+        <v>82</v>
+      </c>
+      <c r="C163" s="11">
+        <v>91</v>
+      </c>
+      <c r="D163" s="11">
+        <v>51</v>
+      </c>
+      <c r="E163" s="11">
+        <v>33</v>
+      </c>
+      <c r="F163" s="11">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A164" s="12">
+        <v>163</v>
+      </c>
+      <c r="B164" s="11">
+        <v>75</v>
+      </c>
+      <c r="C164" s="11">
+        <v>84</v>
+      </c>
+      <c r="D164" s="11">
+        <v>69</v>
+      </c>
+      <c r="E164" s="11">
+        <v>83</v>
+      </c>
+      <c r="F164" s="11">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A165" s="12">
+        <v>164</v>
+      </c>
+      <c r="B165" s="11">
+        <v>88</v>
+      </c>
+      <c r="C165" s="11">
+        <v>90</v>
+      </c>
+      <c r="D165" s="11">
+        <v>76</v>
+      </c>
+      <c r="E165" s="11">
+        <v>49</v>
+      </c>
+      <c r="F165" s="11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A166" s="12">
+        <v>165</v>
+      </c>
+      <c r="B166" s="11">
+        <v>97</v>
+      </c>
+      <c r="C166" s="11">
+        <v>58</v>
+      </c>
+      <c r="D166" s="11">
+        <v>94</v>
+      </c>
+      <c r="E166" s="11">
+        <v>69</v>
+      </c>
+      <c r="F166" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A167" s="12">
+        <v>166</v>
+      </c>
+      <c r="B167" s="11">
+        <v>88</v>
+      </c>
+      <c r="C167" s="11">
+        <v>84</v>
+      </c>
+      <c r="D167" s="11">
+        <v>64</v>
+      </c>
+      <c r="E167" s="11">
+        <v>91</v>
+      </c>
+      <c r="F167" s="11">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A168" s="12">
+        <v>167</v>
+      </c>
+      <c r="B168" s="11">
+        <v>53</v>
+      </c>
+      <c r="C168" s="11">
+        <v>86</v>
+      </c>
+      <c r="D168" s="11">
+        <v>60</v>
+      </c>
+      <c r="E168" s="11">
+        <v>88</v>
+      </c>
+      <c r="F168" s="11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A169" s="12">
+        <v>168</v>
+      </c>
+      <c r="B169" s="11">
+        <v>56</v>
+      </c>
+      <c r="C169" s="11">
+        <v>98</v>
+      </c>
+      <c r="D169" s="11">
+        <v>53</v>
+      </c>
+      <c r="E169" s="11">
+        <v>71</v>
+      </c>
+      <c r="F169" s="11">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A170" s="12">
+        <v>169</v>
+      </c>
+      <c r="B170" s="11">
+        <v>79</v>
+      </c>
+      <c r="C170" s="11">
+        <v>86</v>
+      </c>
+      <c r="D170" s="11">
+        <v>70</v>
+      </c>
+      <c r="E170" s="11">
+        <v>98</v>
+      </c>
+      <c r="F170" s="11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A171" s="12">
+        <v>170</v>
+      </c>
+      <c r="B171" s="11">
+        <v>54</v>
+      </c>
+      <c r="C171" s="11">
+        <v>56</v>
+      </c>
+      <c r="D171" s="11">
+        <v>89</v>
+      </c>
+      <c r="E171" s="11">
+        <v>58</v>
+      </c>
+      <c r="F171" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A172" s="12">
+        <v>171</v>
+      </c>
+      <c r="B172" s="11">
+        <v>69</v>
+      </c>
+      <c r="C172" s="11">
+        <v>89</v>
+      </c>
+      <c r="D172" s="11">
+        <v>95</v>
+      </c>
+      <c r="E172" s="11">
+        <v>97</v>
+      </c>
+      <c r="F172" s="11">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A173" s="12">
+        <v>172</v>
+      </c>
+      <c r="B173" s="11">
+        <v>82</v>
+      </c>
+      <c r="C173" s="11">
+        <v>90</v>
+      </c>
+      <c r="D173" s="11">
+        <v>83</v>
+      </c>
+      <c r="E173" s="11">
+        <v>74</v>
+      </c>
+      <c r="F173" s="11">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A174" s="12">
+        <v>173</v>
+      </c>
+      <c r="B174" s="11">
+        <v>68</v>
+      </c>
+      <c r="C174" s="11">
+        <v>91</v>
+      </c>
+      <c r="D174" s="11">
+        <v>59</v>
+      </c>
+      <c r="E174" s="11">
+        <v>96</v>
+      </c>
+      <c r="F174" s="11">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A175" s="12">
+        <v>174</v>
+      </c>
+      <c r="B175" s="11">
+        <v>96</v>
+      </c>
+      <c r="C175" s="11">
+        <v>75</v>
+      </c>
+      <c r="D175" s="11">
+        <v>80</v>
+      </c>
+      <c r="E175" s="11">
+        <v>42</v>
+      </c>
+      <c r="F175" s="11">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A176" s="12">
+        <v>175</v>
+      </c>
+      <c r="B176" s="11">
+        <v>97</v>
+      </c>
+      <c r="C176" s="11">
+        <v>86</v>
+      </c>
+      <c r="D176" s="11">
+        <v>80</v>
+      </c>
+      <c r="E176" s="11">
+        <v>42</v>
+      </c>
+      <c r="F176" s="11">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A177" s="12">
+        <v>176</v>
+      </c>
+      <c r="B177" s="11">
+        <v>46</v>
+      </c>
+      <c r="C177" s="11">
+        <v>94</v>
+      </c>
+      <c r="D177" s="11">
+        <v>96</v>
+      </c>
+      <c r="E177" s="11">
+        <v>97</v>
+      </c>
+      <c r="F177" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A178" s="12">
+        <v>177</v>
+      </c>
+      <c r="B178" s="11">
+        <v>79</v>
+      </c>
+      <c r="C178" s="11">
+        <v>98</v>
+      </c>
+      <c r="D178" s="11">
+        <v>88</v>
+      </c>
+      <c r="E178" s="11">
+        <v>70</v>
+      </c>
+      <c r="F178" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A179" s="12">
+        <v>178</v>
+      </c>
+      <c r="B179" s="11">
+        <v>21</v>
+      </c>
+      <c r="C179" s="11">
+        <v>75</v>
+      </c>
+      <c r="D179" s="11">
+        <v>93</v>
+      </c>
+      <c r="E179" s="11">
+        <v>83</v>
+      </c>
+      <c r="F179" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A180" s="12">
+        <v>179</v>
+      </c>
+      <c r="B180" s="11">
+        <v>92</v>
+      </c>
+      <c r="C180" s="11">
+        <v>86</v>
+      </c>
+      <c r="D180" s="11">
+        <v>44</v>
+      </c>
+      <c r="E180" s="11">
+        <v>92</v>
+      </c>
+      <c r="F180" s="11">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A181" s="12">
+        <v>180</v>
+      </c>
+      <c r="B181" s="11">
+        <v>42</v>
+      </c>
+      <c r="C181" s="11">
+        <v>91</v>
+      </c>
+      <c r="D181" s="11">
+        <v>90</v>
+      </c>
+      <c r="E181" s="11">
+        <v>36</v>
+      </c>
+      <c r="F181" s="11">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A182" s="12">
+        <v>181</v>
+      </c>
+      <c r="B182" s="11">
+        <v>98</v>
+      </c>
+      <c r="C182" s="11">
+        <v>75</v>
+      </c>
+      <c r="D182" s="11">
+        <v>55</v>
+      </c>
+      <c r="E182" s="11">
+        <v>67</v>
+      </c>
+      <c r="F182" s="11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A183" s="12">
+        <v>182</v>
+      </c>
+      <c r="B183" s="11">
+        <v>97</v>
+      </c>
+      <c r="C183" s="11">
+        <v>90</v>
+      </c>
+      <c r="D183" s="11">
+        <v>66</v>
+      </c>
+      <c r="E183" s="11">
+        <v>95</v>
+      </c>
+      <c r="F183" s="11">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A184" s="12">
+        <v>183</v>
+      </c>
+      <c r="B184" s="11">
+        <v>59</v>
+      </c>
+      <c r="C184" s="11">
+        <v>58</v>
+      </c>
+      <c r="D184" s="11">
+        <v>72</v>
+      </c>
+      <c r="E184" s="11">
+        <v>91</v>
+      </c>
+      <c r="F184" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A185" s="12">
+        <v>184</v>
+      </c>
+      <c r="B185" s="11">
+        <v>69</v>
+      </c>
+      <c r="C185" s="11">
+        <v>90</v>
+      </c>
+      <c r="D185" s="11">
+        <v>68</v>
+      </c>
+      <c r="E185" s="11">
+        <v>66</v>
+      </c>
+      <c r="F185" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A186" s="12">
+        <v>185</v>
+      </c>
+      <c r="B186" s="11">
+        <v>95</v>
+      </c>
+      <c r="C186" s="11">
+        <v>47</v>
+      </c>
+      <c r="D186" s="11">
+        <v>75</v>
+      </c>
+      <c r="E186" s="11">
+        <v>85</v>
+      </c>
+      <c r="F186" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A187" s="12">
+        <v>186</v>
+      </c>
+      <c r="B187" s="11">
+        <v>93</v>
+      </c>
+      <c r="C187" s="11">
+        <v>92</v>
+      </c>
+      <c r="D187" s="11">
+        <v>95</v>
+      </c>
+      <c r="E187" s="11">
+        <v>72</v>
+      </c>
+      <c r="F187" s="11">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A188" s="12">
+        <v>187</v>
+      </c>
+      <c r="B188" s="11">
+        <v>97</v>
+      </c>
+      <c r="C188" s="11">
+        <v>59</v>
+      </c>
+      <c r="D188" s="11">
+        <v>42</v>
+      </c>
+      <c r="E188" s="11">
+        <v>65</v>
+      </c>
+      <c r="F188" s="11">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A189" s="12">
+        <v>188</v>
+      </c>
+      <c r="B189" s="11">
+        <v>18</v>
+      </c>
+      <c r="C189" s="11">
+        <v>95</v>
+      </c>
+      <c r="D189" s="11">
+        <v>94</v>
+      </c>
+      <c r="E189" s="11">
+        <v>42</v>
+      </c>
+      <c r="F189" s="11">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A190" s="12">
+        <v>189</v>
+      </c>
+      <c r="B190" s="11">
+        <v>96</v>
+      </c>
+      <c r="C190" s="11">
+        <v>72</v>
+      </c>
+      <c r="D190" s="11">
+        <v>99</v>
+      </c>
+      <c r="E190" s="11">
+        <v>96</v>
+      </c>
+      <c r="F190" s="11">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A191" s="12">
+        <v>190</v>
+      </c>
+      <c r="B191" s="11">
+        <v>69</v>
+      </c>
+      <c r="C191" s="11">
+        <v>99</v>
+      </c>
+      <c r="D191" s="11">
+        <v>33</v>
+      </c>
+      <c r="E191" s="11">
+        <v>96</v>
+      </c>
+      <c r="F191" s="11">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A192" s="12">
+        <v>191</v>
+      </c>
+      <c r="B192" s="11">
+        <v>31</v>
+      </c>
+      <c r="C192" s="11">
+        <v>80</v>
+      </c>
+      <c r="D192" s="11">
+        <v>67</v>
+      </c>
+      <c r="E192" s="11">
+        <v>87</v>
+      </c>
+      <c r="F192" s="11">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A193" s="12">
+        <v>192</v>
+      </c>
+      <c r="B193" s="11">
+        <v>16</v>
+      </c>
+      <c r="C193" s="11">
+        <v>95</v>
+      </c>
+      <c r="D193" s="11">
+        <v>97</v>
+      </c>
+      <c r="E193" s="11">
+        <v>85</v>
+      </c>
+      <c r="F193" s="11">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A194" s="12">
+        <v>193</v>
+      </c>
+      <c r="B194" s="11">
+        <v>66</v>
+      </c>
+      <c r="C194" s="11">
+        <v>53</v>
+      </c>
+      <c r="D194" s="11">
+        <v>88</v>
+      </c>
+      <c r="E194" s="11">
+        <v>36</v>
+      </c>
+      <c r="F194" s="11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A195" s="12">
+        <v>194</v>
+      </c>
+      <c r="B195" s="11">
+        <v>47</v>
+      </c>
+      <c r="C195" s="11">
+        <v>59</v>
+      </c>
+      <c r="D195" s="11">
+        <v>57</v>
+      </c>
+      <c r="E195" s="11">
+        <v>66</v>
+      </c>
+      <c r="F195" s="11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A196" s="12">
+        <v>195</v>
+      </c>
+      <c r="B196" s="11">
+        <v>77</v>
+      </c>
+      <c r="C196" s="11">
+        <v>85</v>
+      </c>
+      <c r="D196" s="11">
+        <v>99</v>
+      </c>
+      <c r="E196" s="11">
+        <v>92</v>
+      </c>
+      <c r="F196" s="11">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A197" s="12">
+        <v>196</v>
+      </c>
+      <c r="B197" s="11">
+        <v>95</v>
+      </c>
+      <c r="C197" s="11">
+        <v>45</v>
+      </c>
+      <c r="D197" s="11">
+        <v>95</v>
+      </c>
+      <c r="E197" s="11">
+        <v>27</v>
+      </c>
+      <c r="F197" s="11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A198" s="12">
+        <v>197</v>
+      </c>
+      <c r="B198" s="11">
+        <v>55</v>
+      </c>
+      <c r="C198" s="11">
+        <v>86</v>
+      </c>
+      <c r="D198" s="11">
+        <v>120</v>
+      </c>
+      <c r="E198" s="11">
+        <v>98</v>
+      </c>
+      <c r="F198" s="11">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A199" s="12">
+        <v>198</v>
+      </c>
+      <c r="B199" s="11">
+        <v>92</v>
+      </c>
+      <c r="C199" s="11">
+        <v>88</v>
+      </c>
+      <c r="D199" s="11">
+        <v>84</v>
+      </c>
+      <c r="E199" s="11">
+        <v>82</v>
+      </c>
+      <c r="F199" s="11">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A200" s="12">
+        <v>199</v>
+      </c>
+      <c r="B200" s="11">
+        <v>89</v>
+      </c>
+      <c r="C200" s="11">
+        <v>98</v>
+      </c>
+      <c r="D200" s="11">
+        <v>70</v>
+      </c>
+      <c r="E200" s="11">
+        <v>80</v>
+      </c>
+      <c r="F200" s="11"/>
+    </row>
+    <row r="201" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A201" s="12">
+        <v>200</v>
+      </c>
+      <c r="B201" s="11">
+        <v>76</v>
+      </c>
+      <c r="C201" s="11">
+        <v>59</v>
+      </c>
+      <c r="D201" s="11">
+        <v>73</v>
+      </c>
+      <c r="E201" s="11">
+        <v>85</v>
+      </c>
+      <c r="F201" s="11">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A202" s="12">
+        <v>201</v>
+      </c>
+      <c r="B202" s="11">
+        <v>96</v>
+      </c>
+      <c r="C202" s="11">
+        <v>79</v>
+      </c>
+      <c r="D202" s="11">
+        <v>99</v>
+      </c>
+      <c r="E202" s="11">
+        <v>90</v>
+      </c>
+      <c r="F202" s="11">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A203" s="12">
+        <v>202</v>
+      </c>
+      <c r="B203" s="11">
+        <v>70</v>
+      </c>
+      <c r="C203" s="11">
+        <v>82</v>
+      </c>
+      <c r="D203" s="11">
+        <v>82</v>
+      </c>
+      <c r="E203" s="11">
+        <v>94</v>
+      </c>
+      <c r="F203" s="11">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A204" s="12">
+        <v>203</v>
+      </c>
+      <c r="B204" s="11">
+        <v>90</v>
+      </c>
+      <c r="C204" s="11">
+        <v>85</v>
+      </c>
+      <c r="D204" s="11">
+        <v>48</v>
+      </c>
+      <c r="E204" s="11">
+        <v>71</v>
+      </c>
+      <c r="F204" s="11">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A205" s="12">
+        <v>204</v>
+      </c>
+      <c r="B205" s="11">
+        <v>42</v>
+      </c>
+      <c r="C205" s="11">
+        <v>82</v>
+      </c>
+      <c r="D205" s="11">
+        <v>82</v>
+      </c>
+      <c r="E205" s="11">
+        <v>79</v>
+      </c>
+      <c r="F205" s="11">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A206" s="12">
+        <v>205</v>
+      </c>
+      <c r="B206" s="11">
+        <v>51</v>
+      </c>
+      <c r="C206" s="11">
+        <v>13</v>
+      </c>
+      <c r="D206" s="11">
+        <v>65</v>
+      </c>
+      <c r="E206" s="11">
+        <v>59</v>
+      </c>
+      <c r="F206" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A207" s="12">
+        <v>206</v>
+      </c>
+      <c r="B207" s="11">
+        <v>52</v>
+      </c>
+      <c r="C207" s="11">
+        <v>91</v>
+      </c>
+      <c r="D207" s="11">
+        <v>92</v>
+      </c>
+      <c r="E207" s="11">
+        <v>93</v>
+      </c>
+      <c r="F207" s="11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A208" s="12">
+        <v>207</v>
+      </c>
+      <c r="B208" s="11">
+        <v>60</v>
+      </c>
+      <c r="C208" s="11">
+        <v>99</v>
+      </c>
+      <c r="D208" s="11">
+        <v>86</v>
+      </c>
+      <c r="E208" s="11">
+        <v>95</v>
+      </c>
+      <c r="F208" s="11">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A209" s="12">
+        <v>208</v>
+      </c>
+      <c r="B209" s="11">
+        <v>95</v>
+      </c>
+      <c r="C209" s="11">
+        <v>59</v>
+      </c>
+      <c r="D209" s="11">
+        <v>100</v>
+      </c>
+      <c r="E209" s="11">
+        <v>10</v>
+      </c>
+      <c r="F209" s="11">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A210" s="12">
+        <v>209</v>
+      </c>
+      <c r="B210" s="11">
+        <v>52</v>
+      </c>
+      <c r="C210" s="11">
+        <v>55</v>
+      </c>
+      <c r="D210" s="11">
+        <v>83</v>
+      </c>
+      <c r="E210" s="11">
+        <v>96</v>
+      </c>
+      <c r="F210" s="11">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A211" s="12">
+        <v>210</v>
+      </c>
+      <c r="B211" s="11">
+        <v>78</v>
+      </c>
+      <c r="C211" s="11">
+        <v>98</v>
+      </c>
+      <c r="D211" s="11">
+        <v>46</v>
+      </c>
+      <c r="E211" s="11">
+        <v>97</v>
+      </c>
+      <c r="F211" s="11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A212" s="12">
+        <v>211</v>
+      </c>
+      <c r="B212" s="11">
+        <v>84</v>
+      </c>
+      <c r="C212" s="11">
+        <v>90</v>
+      </c>
+      <c r="D212" s="11">
+        <v>83</v>
+      </c>
+      <c r="E212" s="11">
+        <v>35</v>
+      </c>
+      <c r="F212" s="11">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A213" s="12">
+        <v>212</v>
+      </c>
+      <c r="B213" s="11">
+        <v>83</v>
+      </c>
+      <c r="C213" s="11">
+        <v>85</v>
+      </c>
+      <c r="D213" s="11">
+        <v>97</v>
+      </c>
+      <c r="E213" s="11">
+        <v>82</v>
+      </c>
+      <c r="F213" s="11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A214" s="12">
+        <v>213</v>
+      </c>
+      <c r="B214" s="11">
+        <v>61</v>
+      </c>
+      <c r="C214" s="11">
+        <v>92</v>
+      </c>
+      <c r="D214" s="11">
+        <v>30</v>
+      </c>
+      <c r="E214" s="11">
+        <v>96</v>
+      </c>
+      <c r="F214" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A215" s="12">
+        <v>214</v>
+      </c>
+      <c r="B215" s="11">
+        <v>94</v>
+      </c>
+      <c r="C215" s="11">
+        <v>84</v>
+      </c>
+      <c r="D215" s="11">
+        <v>53</v>
+      </c>
+      <c r="E215" s="11">
+        <v>31</v>
+      </c>
+      <c r="F215" s="11">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A216" s="12">
+        <v>215</v>
+      </c>
+      <c r="B216" s="11">
+        <v>88</v>
+      </c>
+      <c r="C216" s="11">
+        <v>63</v>
+      </c>
+      <c r="D216" s="11">
+        <v>91</v>
+      </c>
+      <c r="E216" s="11">
+        <v>69</v>
+      </c>
+      <c r="F216" s="11">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A217" s="12">
+        <v>216</v>
+      </c>
+      <c r="B217" s="11">
+        <v>82</v>
+      </c>
+      <c r="C217" s="11">
+        <v>92</v>
+      </c>
+      <c r="D217" s="11">
+        <v>96</v>
+      </c>
+      <c r="E217" s="11">
+        <v>97</v>
+      </c>
+      <c r="F217" s="11">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A218" s="12">
+        <v>217</v>
+      </c>
+      <c r="B218" s="11">
+        <v>98</v>
+      </c>
+      <c r="C218" s="11">
+        <v>63</v>
+      </c>
+      <c r="D218" s="11">
+        <v>78</v>
+      </c>
+      <c r="E218" s="11">
+        <v>87</v>
+      </c>
+      <c r="F218" s="11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A220" s="10">
+        <f t="shared" ref="A220:F220" si="0">COUNTBLANK(A2:A218)</f>
+        <v>0</v>
+      </c>
+      <c r="B220" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C220" s="10">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D220" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E220" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F220" s="10">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F218" xr:uid="{7031D5CB-845F-C443-A959-7B57D41E4497}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F0A8EB-69C9-44F3-ABC6-9E739B239D9F}">
   <dimension ref="A1:C112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -15653,7 +20114,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{722DCD43-E3C3-9542-BA2D-732C34ED15CC}">
   <dimension ref="A1:B232"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -17390,7 +21851,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C87FAAC5-7D0D-E849-9085-D0FC89AE714D}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>